<commit_message>
Adding a section on McGonigal to Ethics to counter-balance the games = violence stuff
</commit_message>
<xml_diff>
--- a/T1/GDV5002/Marking/GDV5002_PORT1_Marks_2025.xlsx
+++ b/T1/GDV5002/Marking/GDV5002_PORT1_Marks_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2025_26\T1\GDV5002\Marking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C358FDE4-C297-4540-A3EE-D93B68576411}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB99135D-1364-4C2A-9750-1F735D710A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38290" yWindow="-1890" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="27">
   <si>
     <t>Student Name</t>
   </si>
@@ -103,6 +103,9 @@
   </si>
   <si>
     <t>NS</t>
+  </si>
+  <si>
+    <t>Y</t>
   </si>
 </sst>
 </file>
@@ -194,7 +197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -244,11 +247,11 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -279,6 +282,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -601,7 +607,9 @@
       <c r="C2" s="23">
         <v>14</v>
       </c>
-      <c r="D2" s="23"/>
+      <c r="D2" s="23" t="s">
+        <v>26</v>
+      </c>
       <c r="E2" s="23"/>
       <c r="F2" s="30"/>
     </row>
@@ -615,7 +623,9 @@
       <c r="C3" s="14">
         <v>55</v>
       </c>
-      <c r="D3" s="14"/>
+      <c r="D3" s="14" t="s">
+        <v>26</v>
+      </c>
       <c r="E3" s="14"/>
       <c r="F3" s="28"/>
     </row>
@@ -629,7 +639,9 @@
       <c r="C4" s="8">
         <v>87</v>
       </c>
-      <c r="D4" s="8"/>
+      <c r="D4" s="8" t="s">
+        <v>26</v>
+      </c>
       <c r="E4" s="8"/>
       <c r="F4" s="26"/>
     </row>
@@ -643,7 +655,9 @@
       <c r="C5" s="14">
         <v>59</v>
       </c>
-      <c r="D5" s="14"/>
+      <c r="D5" s="14" t="s">
+        <v>26</v>
+      </c>
       <c r="E5" s="14"/>
       <c r="F5" s="28"/>
     </row>
@@ -657,7 +671,9 @@
       <c r="C6" s="14">
         <v>58</v>
       </c>
-      <c r="D6" s="14"/>
+      <c r="D6" s="14" t="s">
+        <v>26</v>
+      </c>
       <c r="E6" s="14"/>
       <c r="F6" s="25"/>
     </row>
@@ -671,7 +687,9 @@
       <c r="C7" s="8">
         <v>84</v>
       </c>
-      <c r="D7" s="8"/>
+      <c r="D7" s="8" t="s">
+        <v>26</v>
+      </c>
       <c r="E7" s="8"/>
       <c r="F7" s="25"/>
     </row>
@@ -685,7 +703,9 @@
       <c r="C8" s="11">
         <v>65</v>
       </c>
-      <c r="D8" s="11"/>
+      <c r="D8" s="11" t="s">
+        <v>26</v>
+      </c>
       <c r="E8" s="11"/>
       <c r="F8" s="27"/>
     </row>
@@ -699,7 +719,9 @@
       <c r="C9" s="14">
         <v>58</v>
       </c>
-      <c r="D9" s="14"/>
+      <c r="D9" s="14" t="s">
+        <v>26</v>
+      </c>
       <c r="E9" s="14"/>
       <c r="F9" s="28"/>
     </row>
@@ -713,7 +735,9 @@
       <c r="C10" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="33"/>
+      <c r="D10" s="33" t="s">
+        <v>26</v>
+      </c>
       <c r="E10" s="33"/>
       <c r="F10" s="25"/>
     </row>
@@ -727,7 +751,9 @@
       <c r="C11" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="19"/>
+      <c r="D11" s="19" t="s">
+        <v>26</v>
+      </c>
       <c r="E11" s="19"/>
       <c r="F11" s="25"/>
     </row>
@@ -741,7 +767,9 @@
       <c r="C12" s="8">
         <v>84</v>
       </c>
-      <c r="D12" s="8"/>
+      <c r="D12" s="8" t="s">
+        <v>26</v>
+      </c>
       <c r="E12" s="8"/>
       <c r="F12" s="26"/>
     </row>
@@ -755,7 +783,9 @@
       <c r="C13" s="8">
         <v>85</v>
       </c>
-      <c r="D13" s="8"/>
+      <c r="D13" s="8" t="s">
+        <v>26</v>
+      </c>
       <c r="E13" s="8"/>
       <c r="F13" s="26"/>
     </row>
@@ -769,7 +799,9 @@
       <c r="C14" s="11">
         <v>64</v>
       </c>
-      <c r="D14" s="11"/>
+      <c r="D14" s="11" t="s">
+        <v>26</v>
+      </c>
       <c r="E14" s="11"/>
       <c r="F14" s="27"/>
     </row>
@@ -783,7 +815,9 @@
       <c r="C15" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="33"/>
+      <c r="D15" s="33" t="s">
+        <v>26</v>
+      </c>
       <c r="E15" s="33"/>
       <c r="F15" s="25"/>
     </row>
@@ -797,7 +831,9 @@
       <c r="C16" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="D16" s="31"/>
+      <c r="D16" s="33" t="s">
+        <v>26</v>
+      </c>
       <c r="E16" s="31"/>
       <c r="F16" s="25"/>
     </row>
@@ -811,7 +847,9 @@
       <c r="C17" s="15">
         <v>61</v>
       </c>
-      <c r="D17" s="9"/>
+      <c r="D17" s="11" t="s">
+        <v>26</v>
+      </c>
       <c r="E17" s="9"/>
       <c r="F17" s="27"/>
     </row>
@@ -825,7 +863,9 @@
       <c r="C18" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="17"/>
+      <c r="D18" s="19" t="s">
+        <v>26</v>
+      </c>
       <c r="E18" s="17"/>
       <c r="F18" s="25"/>
     </row>
@@ -839,7 +879,9 @@
       <c r="C19" s="16">
         <v>45</v>
       </c>
-      <c r="D19" s="4"/>
+      <c r="D19" s="35" t="s">
+        <v>26</v>
+      </c>
       <c r="E19" s="4"/>
       <c r="F19" s="29"/>
     </row>

</xml_diff>

<commit_message>
Did a little more on Ethics for next week
</commit_message>
<xml_diff>
--- a/T1/GDV5002/Marking/GDV5002_PORT1_Marks_2025.xlsx
+++ b/T1/GDV5002/Marking/GDV5002_PORT1_Marks_2025.xlsx
@@ -1,24 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2025_26\T1\GDV5002\Marking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB99135D-1364-4C2A-9750-1F735D710A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAB370D9-B127-40E6-8FFC-E1B7EEA5278E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="46296" windowHeight="25416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -197,7 +208,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -254,7 +265,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -285,6 +295,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -566,7 +594,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" customWidth="1"/>
@@ -611,7 +639,7 @@
         <v>26</v>
       </c>
       <c r="E2" s="23"/>
-      <c r="F2" s="30"/>
+      <c r="F2" s="29"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
@@ -627,7 +655,7 @@
         <v>26</v>
       </c>
       <c r="E3" s="14"/>
-      <c r="F3" s="28"/>
+      <c r="F3" s="27"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
@@ -643,7 +671,7 @@
         <v>26</v>
       </c>
       <c r="E4" s="8"/>
-      <c r="F4" s="26"/>
+      <c r="F4" s="25"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
@@ -659,7 +687,7 @@
         <v>26</v>
       </c>
       <c r="E5" s="14"/>
-      <c r="F5" s="28"/>
+      <c r="F5" s="27"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
@@ -675,7 +703,7 @@
         <v>26</v>
       </c>
       <c r="E6" s="14"/>
-      <c r="F6" s="25"/>
+      <c r="F6" s="24"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
@@ -691,7 +719,7 @@
         <v>26</v>
       </c>
       <c r="E7" s="8"/>
-      <c r="F7" s="25"/>
+      <c r="F7" s="24"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
@@ -707,7 +735,7 @@
         <v>26</v>
       </c>
       <c r="E8" s="11"/>
-      <c r="F8" s="27"/>
+      <c r="F8" s="26"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
@@ -723,23 +751,23 @@
         <v>26</v>
       </c>
       <c r="E9" s="14"/>
-      <c r="F9" s="28"/>
+      <c r="F9" s="27"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="32">
+      <c r="B10" s="31">
         <v>20234956</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C10" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="33" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="33"/>
-      <c r="F10" s="25"/>
+      <c r="D10" s="32" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="32"/>
+      <c r="F10" s="24"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
@@ -755,7 +783,7 @@
         <v>26</v>
       </c>
       <c r="E11" s="19"/>
-      <c r="F11" s="25"/>
+      <c r="F11" s="24"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
@@ -771,7 +799,7 @@
         <v>26</v>
       </c>
       <c r="E12" s="8"/>
-      <c r="F12" s="26"/>
+      <c r="F12" s="25"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
@@ -787,57 +815,57 @@
         <v>26</v>
       </c>
       <c r="E13" s="8"/>
-      <c r="F13" s="26"/>
+      <c r="F13" s="25"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="7">
         <v>20296493</v>
       </c>
-      <c r="C14" s="11">
-        <v>64</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E14" s="11"/>
-      <c r="F14" s="27"/>
+      <c r="C14" s="8">
+        <v>74</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" s="8"/>
+      <c r="F14" s="25"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="31" t="s">
+      <c r="A15" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="32">
+      <c r="B15" s="31">
         <v>20305402</v>
       </c>
-      <c r="C15" s="33" t="s">
+      <c r="C15" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="33" t="s">
-        <v>26</v>
-      </c>
-      <c r="E15" s="33"/>
-      <c r="F15" s="25"/>
+      <c r="D15" s="32" t="s">
+        <v>26</v>
+      </c>
+      <c r="E15" s="32"/>
+      <c r="F15" s="24"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="32">
+      <c r="B16" s="31">
         <v>20297298</v>
       </c>
-      <c r="C16" s="34" t="s">
+      <c r="C16" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="D16" s="33" t="s">
-        <v>26</v>
-      </c>
-      <c r="E16" s="31"/>
-      <c r="F16" s="25"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D16" s="32" t="s">
+        <v>26</v>
+      </c>
+      <c r="E16" s="30"/>
+      <c r="F16" s="24"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
         <v>20</v>
       </c>
@@ -851,9 +879,9 @@
         <v>26</v>
       </c>
       <c r="E17" s="9"/>
-      <c r="F17" s="27"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F17" s="26"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="17" t="s">
         <v>21</v>
       </c>
@@ -867,9 +895,9 @@
         <v>26</v>
       </c>
       <c r="E18" s="17"/>
-      <c r="F18" s="25"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F18" s="24"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>22</v>
       </c>
@@ -879,29 +907,55 @@
       <c r="C19" s="16">
         <v>45</v>
       </c>
-      <c r="D19" s="35" t="s">
+      <c r="D19" s="34" t="s">
         <v>26</v>
       </c>
       <c r="E19" s="4"/>
-      <c r="F19" s="29"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F19" s="28"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B20" s="3"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="3"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="24"/>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="35">
+        <f xml:space="preserve"> 5</f>
+        <v>5</v>
+      </c>
+      <c r="B21" s="15">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="C21" s="38">
+        <f>4</f>
+        <v>4</v>
+      </c>
+      <c r="D21" s="16">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="E21" s="39">
+        <v>1</v>
+      </c>
+      <c r="F21" s="33">
+        <v>3</v>
+      </c>
+      <c r="G21" s="40">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="37"/>
       <c r="B22" s="3"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="36"/>
       <c r="B23" s="3"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="36"/>
       <c r="B24" s="3"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B25" s="3"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Completed GDV5002 marking and updated Excel sheet of overall marks
</commit_message>
<xml_diff>
--- a/T1/GDV5002/Marking/GDV5002_PORT1_Marks_2025.xlsx
+++ b/T1/GDV5002/Marking/GDV5002_PORT1_Marks_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2025_26\T1\GDV5002\Marking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B7665D7-413F-4FE0-9966-8ECE481DB4C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7B7CB94-451E-497A-98DC-F10EF51EF59A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="4344" windowWidth="38376" windowHeight="20856" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="35">
   <si>
     <t>Student Name</t>
   </si>
@@ -138,6 +138,9 @@
   </si>
   <si>
     <t xml:space="preserve">Number of Students </t>
+  </si>
+  <si>
+    <t>Deferral/Resit Mark</t>
   </si>
 </sst>
 </file>
@@ -229,7 +232,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -332,17 +335,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -637,9 +633,10 @@
     <col min="4" max="4" width="14.109375" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="13.5546875" customWidth="1"/>
+    <col min="7" max="7" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -658,8 +655,11 @@
       <c r="F1" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G1" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="21" t="s">
         <v>5</v>
       </c>
@@ -676,8 +676,11 @@
         <v>14</v>
       </c>
       <c r="F2" s="29"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G2" s="39">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
         <v>6</v>
       </c>
@@ -694,8 +697,9 @@
         <v>55</v>
       </c>
       <c r="F3" s="27"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G3" s="36"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>7</v>
       </c>
@@ -712,8 +716,9 @@
         <v>87</v>
       </c>
       <c r="F4" s="25"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G4" s="36"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
         <v>8</v>
       </c>
@@ -730,8 +735,9 @@
         <v>59</v>
       </c>
       <c r="F5" s="27"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G5" s="36"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
         <v>9</v>
       </c>
@@ -748,8 +754,9 @@
         <v>58</v>
       </c>
       <c r="F6" s="24"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G6" s="36"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
@@ -766,8 +773,9 @@
         <v>84</v>
       </c>
       <c r="F7" s="24"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G7" s="36"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>11</v>
       </c>
@@ -784,8 +792,9 @@
         <v>65</v>
       </c>
       <c r="F8" s="26"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G8" s="36"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
         <v>12</v>
       </c>
@@ -802,8 +811,9 @@
         <v>58</v>
       </c>
       <c r="F9" s="27"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G9" s="36"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="30" t="s">
         <v>13</v>
       </c>
@@ -820,8 +830,11 @@
         <v>23</v>
       </c>
       <c r="F10" s="24"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G10" s="20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
         <v>14</v>
       </c>
@@ -838,8 +851,9 @@
         <v>25</v>
       </c>
       <c r="F11" s="24"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G11" s="36"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>15</v>
       </c>
@@ -856,8 +870,9 @@
         <v>84</v>
       </c>
       <c r="F12" s="25"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G12" s="36"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>16</v>
       </c>
@@ -874,8 +889,9 @@
         <v>85</v>
       </c>
       <c r="F13" s="25"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G13" s="36"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>17</v>
       </c>
@@ -892,8 +908,9 @@
         <v>74</v>
       </c>
       <c r="F14" s="25"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G14" s="36"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="30" t="s">
         <v>18</v>
       </c>
@@ -910,8 +927,11 @@
         <v>23</v>
       </c>
       <c r="F15" s="24"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G15" s="20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="30" t="s">
         <v>19</v>
       </c>
@@ -928,6 +948,9 @@
         <v>23</v>
       </c>
       <c r="F16" s="24"/>
+      <c r="G16" s="38">
+        <v>50</v>
+      </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
@@ -946,6 +969,7 @@
         <v>61</v>
       </c>
       <c r="F17" s="26"/>
+      <c r="G17" s="36"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="17" t="s">
@@ -964,6 +988,7 @@
         <v>25</v>
       </c>
       <c r="F18" s="24"/>
+      <c r="G18" s="36"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
@@ -982,41 +1007,36 @@
         <v>45</v>
       </c>
       <c r="F19" s="28"/>
+      <c r="G19" s="36"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="40"/>
-      <c r="B20" s="41"/>
-      <c r="C20" s="42"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="40"/>
-      <c r="F20" s="44"/>
+      <c r="B20" s="40"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="41"/>
+      <c r="F20" s="24"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="40"/>
-      <c r="B21" s="41"/>
-      <c r="C21" s="42"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="44"/>
+      <c r="B21" s="40"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="41"/>
+      <c r="F21" s="24"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="40" t="s">
+      <c r="A22" t="s">
         <v>33</v>
       </c>
-      <c r="B22" s="41">
+      <c r="B22" s="40">
         <v>18</v>
       </c>
-      <c r="C22" s="42"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="40"/>
-      <c r="F22" s="44"/>
-      <c r="G22" s="40"/>
+      <c r="C22" s="36"/>
+      <c r="D22" s="41"/>
+      <c r="F22" s="24"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="45" t="s">
+      <c r="B23" s="42" t="s">
         <v>28</v>
       </c>
       <c r="C23" s="38" t="s">
@@ -1045,8 +1065,8 @@
         <v>2</v>
       </c>
       <c r="C24" s="38">
-        <f>4</f>
-        <v>4</v>
+        <f>5</f>
+        <v>5</v>
       </c>
       <c r="D24" s="16">
         <f>1</f>
@@ -1059,7 +1079,7 @@
         <v>3</v>
       </c>
       <c r="G24" s="20">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>